<commit_message>
Updating hydro power costs, adding cutoff treshhold for smallest written timeseries values.
</commit_message>
<xml_diff>
--- a/src_files/data_files/hydroUpd-v1.xlsx
+++ b/src_files/data_files/hydroUpd-v1.xlsx
@@ -1,22 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BB\bb-master\north_european_model\src_files\data_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{380D2174-13BF-4722-8CF4-7C5D3819AC03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA340D2A-A1DA-4DBA-87D2-E2C2D43A749C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="747" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="747" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nodedata" sheetId="13" r:id="rId1"/>
     <sheet name="unitdata" sheetId="14" r:id="rId2"/>
     <sheet name="userconstraintdata" sheetId="17" r:id="rId3"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -38,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="112">
   <si>
     <t>AT00</t>
   </si>
@@ -344,13 +348,43 @@
   </si>
   <si>
     <t>nodeBalance</t>
+  </si>
+  <si>
+    <t>vomCosts</t>
+  </si>
+  <si>
+    <t>GDP pc of country</t>
+  </si>
+  <si>
+    <t>vomCosts country multiplier</t>
+  </si>
+  <si>
+    <t>region multiplier</t>
+  </si>
+  <si>
+    <t>final</t>
+  </si>
+  <si>
+    <t>DKE1</t>
+  </si>
+  <si>
+    <t>DKW1</t>
+  </si>
+  <si>
+    <t>EE00</t>
+  </si>
+  <si>
+    <t>rampUpCost</t>
+  </si>
+  <si>
+    <t>rampDownCost</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -413,6 +447,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="10">
@@ -530,12 +571,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -589,14 +631,28 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{FC31EDF3-2535-4BD0-9B77-3909C39E0667}"/>
     <cellStyle name="Normal 4" xfId="1" xr:uid="{F009F437-1BF9-4014-B677-DDB3856DFBE9}"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="10">
     <dxf>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -616,7 +672,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="3" formatCode="#,##0"/>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -666,6 +721,1422 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="vomcost mult"/>
+      <sheetName val="VRE-NT2030"/>
+      <sheetName val="wind"/>
+      <sheetName val="onshore"/>
+      <sheetName val="offshore"/>
+      <sheetName val="PV"/>
+      <sheetName val="VRE summary"/>
+      <sheetName val="unitdata_VRE"/>
+      <sheetName val="battery cap eurostat"/>
+      <sheetName val="battery scen SPE"/>
+      <sheetName val="battery summary"/>
+      <sheetName val="unitdata_battery"/>
+      <sheetName val="unitdata_nuclearThermal"/>
+      <sheetName val="unitdata_demandRed"/>
+      <sheetName val="transferdata"/>
+      <sheetName val="emissiondata"/>
+      <sheetName val="nodedata"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="11">
+          <cell r="O11">
+            <v>45140</v>
+          </cell>
+          <cell r="P11">
+            <v>0.12757648618174755</v>
+          </cell>
+          <cell r="Q11">
+            <v>1</v>
+          </cell>
+          <cell r="R11">
+            <v>0.128</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="O12">
+            <v>44440</v>
+          </cell>
+          <cell r="P12">
+            <v>0.12078898170883434</v>
+          </cell>
+          <cell r="Q12">
+            <v>1</v>
+          </cell>
+          <cell r="R12">
+            <v>0.121</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="O13">
+            <v>96081</v>
+          </cell>
+          <cell r="P13">
+            <v>0.4556524459454061</v>
+          </cell>
+          <cell r="Q13">
+            <v>1</v>
+          </cell>
+          <cell r="R13">
+            <v>0.45600000000000002</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="O14">
+            <v>43110</v>
+          </cell>
+          <cell r="P14">
+            <v>0.1075929542938924</v>
+          </cell>
+          <cell r="Q14">
+            <v>1</v>
+          </cell>
+          <cell r="R14">
+            <v>0.108</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="O15">
+            <v>58160</v>
+          </cell>
+          <cell r="P15">
+            <v>0.2376393292909858</v>
+          </cell>
+          <cell r="Q15">
+            <v>1.05</v>
+          </cell>
+          <cell r="R15">
+            <v>0.25</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="O16">
+            <v>58160</v>
+          </cell>
+          <cell r="P16">
+            <v>0.2376393292909858</v>
+          </cell>
+          <cell r="Q16">
+            <v>1</v>
+          </cell>
+          <cell r="R16">
+            <v>0.23799999999999999</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="O17">
+            <v>21060</v>
+          </cell>
+          <cell r="P17">
+            <v>-0.20352670171052795</v>
+          </cell>
+          <cell r="Q17">
+            <v>1</v>
+          </cell>
+          <cell r="R17">
+            <v>-0.20399999999999999</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="O18">
+            <v>27800</v>
+          </cell>
+          <cell r="P18">
+            <v>-8.2940272641919402E-2</v>
+          </cell>
+          <cell r="Q18">
+            <v>1</v>
+          </cell>
+          <cell r="R18">
+            <v>-8.3000000000000004E-2</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="O19">
+            <v>43110</v>
+          </cell>
+          <cell r="P19">
+            <v>0.1075929542938924</v>
+          </cell>
+          <cell r="Q19">
+            <v>1</v>
+          </cell>
+          <cell r="R19">
+            <v>0.108</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="O20">
+            <v>38110</v>
+          </cell>
+          <cell r="P20">
+            <v>5.4053880212171543E-2</v>
+          </cell>
+          <cell r="Q20">
+            <v>1</v>
+          </cell>
+          <cell r="R20">
+            <v>5.3999999999999999E-2</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="O21">
+            <v>19690</v>
+          </cell>
+          <cell r="P21">
+            <v>-0.2327393524218774</v>
+          </cell>
+          <cell r="Q21">
+            <v>1</v>
+          </cell>
+          <cell r="R21">
+            <v>-0.23300000000000001</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="O22">
+            <v>16910</v>
+          </cell>
+          <cell r="P22">
+            <v>-0.29884146096225389</v>
+          </cell>
+          <cell r="Q22">
+            <v>1</v>
+          </cell>
+          <cell r="R22">
+            <v>-0.29899999999999999</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="O23">
+            <v>50880</v>
+          </cell>
+          <cell r="P23">
+            <v>0.17956203408036178</v>
+          </cell>
+          <cell r="Q23">
+            <v>1</v>
+          </cell>
+          <cell r="R23">
+            <v>0.18</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="O24">
+            <v>66460</v>
+          </cell>
+          <cell r="P24">
+            <v>0.2955752683826966</v>
+          </cell>
+          <cell r="Q24">
+            <v>1.05</v>
+          </cell>
+          <cell r="R24">
+            <v>0.31</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="O25">
+            <v>66460</v>
+          </cell>
+          <cell r="P25">
+            <v>0.2955752683826966</v>
+          </cell>
+          <cell r="Q25">
+            <v>1.1000000000000001</v>
+          </cell>
+          <cell r="R25">
+            <v>0.32500000000000001</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="O26">
+            <v>66460</v>
+          </cell>
+          <cell r="P26">
+            <v>0.2955752683826966</v>
+          </cell>
+          <cell r="Q26">
+            <v>1</v>
+          </cell>
+          <cell r="R26">
+            <v>0.29599999999999999</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="O27">
+            <v>16470</v>
+          </cell>
+          <cell r="P27">
+            <v>-0.31029146939024133</v>
+          </cell>
+          <cell r="Q27">
+            <v>1</v>
+          </cell>
+          <cell r="R27">
+            <v>-0.31</v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="O28">
+            <v>48310</v>
+          </cell>
+          <cell r="P28">
+            <v>0.15705196892652412</v>
+          </cell>
+          <cell r="Q28">
+            <v>1.1499999999999999</v>
+          </cell>
+          <cell r="R28">
+            <v>0.18099999999999999</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="O29">
+            <v>48310</v>
+          </cell>
+          <cell r="P29">
+            <v>0.15705196892652412</v>
+          </cell>
+          <cell r="Q29">
+            <v>1.1000000000000001</v>
+          </cell>
+          <cell r="R29">
+            <v>0.17299999999999999</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="O30">
+            <v>48310</v>
+          </cell>
+          <cell r="P30">
+            <v>0.15705196892652412</v>
+          </cell>
+          <cell r="Q30">
+            <v>1.05</v>
+          </cell>
+          <cell r="R30">
+            <v>0.16500000000000001</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="O31">
+            <v>48310</v>
+          </cell>
+          <cell r="P31">
+            <v>0.15705196892652412</v>
+          </cell>
+          <cell r="Q31">
+            <v>1</v>
+          </cell>
+          <cell r="R31">
+            <v>0.157</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="O32">
+            <v>49193</v>
+          </cell>
+          <cell r="P32">
+            <v>0.16491823994601576</v>
+          </cell>
+          <cell r="Q32">
+            <v>1</v>
+          </cell>
+          <cell r="R32">
+            <v>0.16500000000000001</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
+      <sheetData sheetId="15" refreshError="1"/>
+      <sheetData sheetId="16" refreshError="1"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="unittypedata"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="1">
+          <cell r="C1" t="str">
+            <v>Generator_ID</v>
+          </cell>
+          <cell r="S1" t="str">
+            <v>vomCosts</v>
+          </cell>
+          <cell r="Y1" t="str">
+            <v>rampUpCost</v>
+          </cell>
+          <cell r="Z1" t="str">
+            <v>rampDownCost</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="C3" t="str">
+            <v>Onshore Wind</v>
+          </cell>
+          <cell r="S3">
+            <v>1</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="C4" t="str">
+            <v>Offshore Wind</v>
+          </cell>
+          <cell r="S4">
+            <v>1.5</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="C5" t="str">
+            <v>Solar PV</v>
+          </cell>
+          <cell r="S5">
+            <v>0.5</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="C7" t="str">
+            <v>Run-of-River</v>
+          </cell>
+          <cell r="S7">
+            <v>2.2000000000000002</v>
+          </cell>
+          <cell r="Y7">
+            <v>5.5</v>
+          </cell>
+          <cell r="Z7">
+            <v>5.5</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="C8" t="str">
+            <v>Reservoir</v>
+          </cell>
+          <cell r="S8">
+            <v>2</v>
+          </cell>
+          <cell r="Y8">
+            <v>5</v>
+          </cell>
+          <cell r="Z8">
+            <v>5</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="C9" t="str">
+            <v>PS Open turbine</v>
+          </cell>
+          <cell r="S9">
+            <v>1.5</v>
+          </cell>
+          <cell r="Y9">
+            <v>4</v>
+          </cell>
+          <cell r="Z9">
+            <v>4</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="C10" t="str">
+            <v>PS Open pump</v>
+          </cell>
+          <cell r="S10">
+            <v>1.4</v>
+          </cell>
+          <cell r="Y10">
+            <v>3.5</v>
+          </cell>
+          <cell r="Z10">
+            <v>3.5</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="C11" t="str">
+            <v>PS Closed turbine</v>
+          </cell>
+          <cell r="S11">
+            <v>1.1000000000000001</v>
+          </cell>
+          <cell r="Y11">
+            <v>3.1</v>
+          </cell>
+          <cell r="Z11">
+            <v>3.1</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="C12" t="str">
+            <v>PS Closed pump</v>
+          </cell>
+          <cell r="S12">
+            <v>1</v>
+          </cell>
+          <cell r="Y12">
+            <v>3</v>
+          </cell>
+          <cell r="Z12">
+            <v>3</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="C14" t="str">
+            <v>Oil shale old</v>
+          </cell>
+          <cell r="S14">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y14">
+            <v>44</v>
+          </cell>
+          <cell r="Z14">
+            <v>44</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="C15" t="str">
+            <v>Oil shale new Bio</v>
+          </cell>
+          <cell r="S15">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y15">
+            <v>28.6</v>
+          </cell>
+          <cell r="Z15">
+            <v>28.6</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="C16" t="str">
+            <v>Oil shale new</v>
+          </cell>
+          <cell r="S16">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y16">
+            <v>28.6</v>
+          </cell>
+          <cell r="Z16">
+            <v>28.6</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="C17" t="str">
+            <v>Lignite old 2 Bio</v>
+          </cell>
+          <cell r="S17">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y17">
+            <v>40.700000000000003</v>
+          </cell>
+          <cell r="Z17">
+            <v>40.700000000000003</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="C18" t="str">
+            <v>Lignite old 2</v>
+          </cell>
+          <cell r="S18">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y18">
+            <v>40.700000000000003</v>
+          </cell>
+          <cell r="Z18">
+            <v>40.700000000000003</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="C19" t="str">
+            <v>Lignite old 1 Bio</v>
+          </cell>
+          <cell r="S19">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y19">
+            <v>47</v>
+          </cell>
+          <cell r="Z19">
+            <v>47</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="C20" t="str">
+            <v>Lignite old 1</v>
+          </cell>
+          <cell r="S20">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y20">
+            <v>47</v>
+          </cell>
+          <cell r="Z20">
+            <v>47</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="C21" t="str">
+            <v>Lignite new</v>
+          </cell>
+          <cell r="S21">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y21">
+            <v>28.6</v>
+          </cell>
+          <cell r="Z21">
+            <v>28.6</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="C22" t="str">
+            <v>Lignite CCS</v>
+          </cell>
+          <cell r="S22">
+            <v>6.6</v>
+          </cell>
+          <cell r="Y22">
+            <v>40.700000000000003</v>
+          </cell>
+          <cell r="Z22">
+            <v>40.700000000000003</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="C23" t="str">
+            <v>Light oil</v>
+          </cell>
+          <cell r="S23">
+            <v>1.1000000000000001</v>
+          </cell>
+          <cell r="Y23">
+            <v>19.2</v>
+          </cell>
+          <cell r="Z23">
+            <v>19.2</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="C24" t="str">
+            <v>Heavy oil old 2</v>
+          </cell>
+          <cell r="S24">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y24">
+            <v>40.700000000000003</v>
+          </cell>
+          <cell r="Z24">
+            <v>40.700000000000003</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="C25" t="str">
+            <v>Heavy oil old 1</v>
+          </cell>
+          <cell r="S25">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y25">
+            <v>47</v>
+          </cell>
+          <cell r="Z25">
+            <v>47</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="C26" t="str">
+            <v>Heavy oil old 1 Bio</v>
+          </cell>
+          <cell r="S26">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y26">
+            <v>40.700000000000003</v>
+          </cell>
+          <cell r="Z26">
+            <v>40.700000000000003</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="C27" t="str">
+            <v>Hard coal old 1 Bio</v>
+          </cell>
+          <cell r="S27">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y27">
+            <v>47</v>
+          </cell>
+          <cell r="Z27">
+            <v>47</v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="C28" t="str">
+            <v>Hard coal old 2 Bio</v>
+          </cell>
+          <cell r="S28">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y28">
+            <v>40.700000000000003</v>
+          </cell>
+          <cell r="Z28">
+            <v>40.700000000000003</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="C29" t="str">
+            <v>Hard coal old 2</v>
+          </cell>
+          <cell r="S29">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y29">
+            <v>40.700000000000003</v>
+          </cell>
+          <cell r="Z29">
+            <v>40.700000000000003</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="C30" t="str">
+            <v>Hard coal old 1</v>
+          </cell>
+          <cell r="S30">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y30">
+            <v>47</v>
+          </cell>
+          <cell r="Z30">
+            <v>47</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="C31" t="str">
+            <v>Hard coal new Bio</v>
+          </cell>
+          <cell r="S31">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y31">
+            <v>28.6</v>
+          </cell>
+          <cell r="Z31">
+            <v>28.6</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="C32" t="str">
+            <v>Hard coal new</v>
+          </cell>
+          <cell r="S32">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y32">
+            <v>28.6</v>
+          </cell>
+          <cell r="Z32">
+            <v>28.6</v>
+          </cell>
+        </row>
+        <row r="33">
+          <cell r="C33" t="str">
+            <v>Gas conventional old 2 Bio</v>
+          </cell>
+          <cell r="S33">
+            <v>1.1000000000000001</v>
+          </cell>
+          <cell r="Y33">
+            <v>29.4</v>
+          </cell>
+          <cell r="Z33">
+            <v>29.4</v>
+          </cell>
+        </row>
+        <row r="34">
+          <cell r="C34" t="str">
+            <v>Gas conventional old 2</v>
+          </cell>
+          <cell r="S34">
+            <v>1.1000000000000001</v>
+          </cell>
+          <cell r="Y34">
+            <v>29.4</v>
+          </cell>
+          <cell r="Z34">
+            <v>29.4</v>
+          </cell>
+        </row>
+        <row r="35">
+          <cell r="C35" t="str">
+            <v>Gas conventional old 1</v>
+          </cell>
+          <cell r="S35">
+            <v>1.1000000000000001</v>
+          </cell>
+          <cell r="Y35">
+            <v>34.799999999999997</v>
+          </cell>
+          <cell r="Z35">
+            <v>34.799999999999997</v>
+          </cell>
+        </row>
+        <row r="36">
+          <cell r="C36" t="str">
+            <v>Gas OCGT old</v>
+          </cell>
+          <cell r="S36">
+            <v>1.6</v>
+          </cell>
+          <cell r="Y36">
+            <v>26.2</v>
+          </cell>
+          <cell r="Z36">
+            <v>26.2</v>
+          </cell>
+        </row>
+        <row r="37">
+          <cell r="C37" t="str">
+            <v>Gas OCGT new</v>
+          </cell>
+          <cell r="S37">
+            <v>1.6</v>
+          </cell>
+          <cell r="Y37">
+            <v>12.1</v>
+          </cell>
+          <cell r="Z37">
+            <v>12.1</v>
+          </cell>
+        </row>
+        <row r="38">
+          <cell r="C38" t="str">
+            <v>Gas CCGT present 2</v>
+          </cell>
+          <cell r="S38">
+            <v>1.6</v>
+          </cell>
+          <cell r="Y38">
+            <v>18</v>
+          </cell>
+          <cell r="Z38">
+            <v>18</v>
+          </cell>
+        </row>
+        <row r="39">
+          <cell r="C39" t="str">
+            <v>Gas CCGT present 1</v>
+          </cell>
+          <cell r="S39">
+            <v>1.6</v>
+          </cell>
+          <cell r="Y39">
+            <v>18</v>
+          </cell>
+          <cell r="Z39">
+            <v>18</v>
+          </cell>
+        </row>
+        <row r="40">
+          <cell r="C40" t="str">
+            <v>Gas CCGT old 2 Bio</v>
+          </cell>
+          <cell r="S40">
+            <v>1.6</v>
+          </cell>
+          <cell r="Y40">
+            <v>30.9</v>
+          </cell>
+          <cell r="Z40">
+            <v>30.9</v>
+          </cell>
+        </row>
+        <row r="41">
+          <cell r="C41" t="str">
+            <v>Gas CCGT old 2</v>
+          </cell>
+          <cell r="S41">
+            <v>1.6</v>
+          </cell>
+          <cell r="Y41">
+            <v>30.9</v>
+          </cell>
+          <cell r="Z41">
+            <v>30.9</v>
+          </cell>
+        </row>
+        <row r="42">
+          <cell r="C42" t="str">
+            <v>Gas CCGT old 1</v>
+          </cell>
+          <cell r="S42">
+            <v>1.6</v>
+          </cell>
+          <cell r="Y42">
+            <v>39.5</v>
+          </cell>
+          <cell r="Z42">
+            <v>39.5</v>
+          </cell>
+        </row>
+        <row r="43">
+          <cell r="C43" t="str">
+            <v>Gas CCGT new</v>
+          </cell>
+          <cell r="S43">
+            <v>1.6</v>
+          </cell>
+          <cell r="Y43">
+            <v>18</v>
+          </cell>
+          <cell r="Z43">
+            <v>18</v>
+          </cell>
+        </row>
+        <row r="45">
+          <cell r="C45" t="str">
+            <v>Hard coal CCS</v>
+          </cell>
+          <cell r="S45">
+            <v>6.6</v>
+          </cell>
+          <cell r="Y45">
+            <v>40.700000000000003</v>
+          </cell>
+          <cell r="Z45">
+            <v>40.700000000000003</v>
+          </cell>
+        </row>
+        <row r="46">
+          <cell r="C46" t="str">
+            <v>Gas CCGT CCS</v>
+          </cell>
+          <cell r="S46">
+            <v>3.2</v>
+          </cell>
+          <cell r="Y46">
+            <v>30.9</v>
+          </cell>
+          <cell r="Z46">
+            <v>30.9</v>
+          </cell>
+        </row>
+        <row r="48">
+          <cell r="C48" t="str">
+            <v>Nuclear</v>
+          </cell>
+          <cell r="S48">
+            <v>3</v>
+          </cell>
+          <cell r="Y48">
+            <v>60</v>
+          </cell>
+          <cell r="Z48">
+            <v>240</v>
+          </cell>
+        </row>
+        <row r="49">
+          <cell r="C49" t="str">
+            <v>Nuclear-flex</v>
+          </cell>
+          <cell r="S49">
+            <v>3.1</v>
+          </cell>
+          <cell r="Y49">
+            <v>5</v>
+          </cell>
+          <cell r="Z49">
+            <v>45</v>
+          </cell>
+        </row>
+        <row r="51">
+          <cell r="C51" t="str">
+            <v>Industry renewable CHP</v>
+          </cell>
+          <cell r="S51">
+            <v>2</v>
+          </cell>
+          <cell r="Y51">
+            <v>42.5</v>
+          </cell>
+          <cell r="Z51">
+            <v>42.5</v>
+          </cell>
+        </row>
+        <row r="52">
+          <cell r="C52" t="str">
+            <v>Industry non-renewable CHP</v>
+          </cell>
+          <cell r="S52">
+            <v>2</v>
+          </cell>
+          <cell r="Y52">
+            <v>47.5</v>
+          </cell>
+          <cell r="Z52">
+            <v>47.5</v>
+          </cell>
+        </row>
+        <row r="53">
+          <cell r="C53" t="str">
+            <v>Industry gas CHP</v>
+          </cell>
+          <cell r="S53">
+            <v>2</v>
+          </cell>
+          <cell r="Y53">
+            <v>47.5</v>
+          </cell>
+          <cell r="Z53">
+            <v>47.5</v>
+          </cell>
+        </row>
+        <row r="55">
+          <cell r="C55" t="str">
+            <v>Battery discharger 4h</v>
+          </cell>
+          <cell r="S55">
+            <v>1.2</v>
+          </cell>
+        </row>
+        <row r="56">
+          <cell r="C56" t="str">
+            <v>Battery discharger</v>
+          </cell>
+          <cell r="S56">
+            <v>1</v>
+          </cell>
+        </row>
+        <row r="57">
+          <cell r="C57" t="str">
+            <v>Battery charger 4h</v>
+          </cell>
+          <cell r="S57">
+            <v>1.2</v>
+          </cell>
+        </row>
+        <row r="58">
+          <cell r="C58" t="str">
+            <v>Battery charger</v>
+          </cell>
+          <cell r="S58">
+            <v>1</v>
+          </cell>
+        </row>
+        <row r="60">
+          <cell r="C60" t="str">
+            <v>Solar Thermal</v>
+          </cell>
+        </row>
+        <row r="61">
+          <cell r="C61" t="str">
+            <v>Ground source heat pump</v>
+          </cell>
+          <cell r="S61">
+            <v>6</v>
+          </cell>
+        </row>
+        <row r="62">
+          <cell r="C62" t="str">
+            <v>Waste HOB</v>
+          </cell>
+          <cell r="S62">
+            <v>2</v>
+          </cell>
+          <cell r="Y62">
+            <v>20</v>
+          </cell>
+          <cell r="Z62">
+            <v>20</v>
+          </cell>
+        </row>
+        <row r="63">
+          <cell r="C63" t="str">
+            <v>Oil HOB</v>
+          </cell>
+          <cell r="S63">
+            <v>2</v>
+          </cell>
+          <cell r="Y63">
+            <v>20</v>
+          </cell>
+          <cell r="Z63">
+            <v>20</v>
+          </cell>
+        </row>
+        <row r="64">
+          <cell r="C64" t="str">
+            <v>Gas HOB</v>
+          </cell>
+          <cell r="S64">
+            <v>2</v>
+          </cell>
+          <cell r="Y64">
+            <v>20</v>
+          </cell>
+          <cell r="Z64">
+            <v>20</v>
+          </cell>
+        </row>
+        <row r="65">
+          <cell r="C65" t="str">
+            <v>Bio HOB</v>
+          </cell>
+          <cell r="S65">
+            <v>2</v>
+          </cell>
+          <cell r="Y65">
+            <v>20</v>
+          </cell>
+          <cell r="Z65">
+            <v>20</v>
+          </cell>
+        </row>
+        <row r="66">
+          <cell r="C66" t="str">
+            <v>Electric boiler</v>
+          </cell>
+          <cell r="S66">
+            <v>13</v>
+          </cell>
+        </row>
+        <row r="67">
+          <cell r="C67" t="str">
+            <v>Waste CHP</v>
+          </cell>
+          <cell r="S67">
+            <v>2</v>
+          </cell>
+          <cell r="Y67">
+            <v>75</v>
+          </cell>
+          <cell r="Z67">
+            <v>75</v>
+          </cell>
+        </row>
+        <row r="68">
+          <cell r="C68" t="str">
+            <v>Coal CHP</v>
+          </cell>
+          <cell r="S68">
+            <v>2</v>
+          </cell>
+          <cell r="Y68">
+            <v>75</v>
+          </cell>
+          <cell r="Z68">
+            <v>75</v>
+          </cell>
+        </row>
+        <row r="69">
+          <cell r="C69" t="str">
+            <v>Bio CHP</v>
+          </cell>
+          <cell r="S69">
+            <v>2</v>
+          </cell>
+          <cell r="Y69">
+            <v>45</v>
+          </cell>
+          <cell r="Z69">
+            <v>45</v>
+          </cell>
+        </row>
+        <row r="70">
+          <cell r="C70" t="str">
+            <v>Gas CCGT CHP</v>
+          </cell>
+          <cell r="S70">
+            <v>1.6</v>
+          </cell>
+          <cell r="Y70">
+            <v>18</v>
+          </cell>
+          <cell r="Z70">
+            <v>18</v>
+          </cell>
+        </row>
+        <row r="71">
+          <cell r="C71" t="str">
+            <v>Coal HOB</v>
+          </cell>
+          <cell r="S71">
+            <v>2</v>
+          </cell>
+        </row>
+        <row r="72">
+          <cell r="C72" t="str">
+            <v>Coal CHP extraction</v>
+          </cell>
+          <cell r="S72">
+            <v>2</v>
+          </cell>
+          <cell r="Y72">
+            <v>75</v>
+          </cell>
+          <cell r="Z72">
+            <v>75</v>
+          </cell>
+        </row>
+        <row r="73">
+          <cell r="C73" t="str">
+            <v>Bio CHP extraction</v>
+          </cell>
+          <cell r="S73">
+            <v>2</v>
+          </cell>
+          <cell r="Y73">
+            <v>45</v>
+          </cell>
+          <cell r="Z73">
+            <v>45</v>
+          </cell>
+        </row>
+        <row r="74">
+          <cell r="C74" t="str">
+            <v>Gas CHP extraction</v>
+          </cell>
+          <cell r="S74">
+            <v>1.6</v>
+          </cell>
+          <cell r="Y74">
+            <v>18</v>
+          </cell>
+          <cell r="Z74">
+            <v>18</v>
+          </cell>
+        </row>
+        <row r="75">
+          <cell r="C75" t="str">
+            <v>Oil shale CHP</v>
+          </cell>
+          <cell r="S75">
+            <v>3.3</v>
+          </cell>
+          <cell r="Y75">
+            <v>28.6</v>
+          </cell>
+          <cell r="Z75">
+            <v>28.6</v>
+          </cell>
+        </row>
+        <row r="76">
+          <cell r="C76" t="str">
+            <v>Gas OCGT CHP</v>
+          </cell>
+          <cell r="S76">
+            <v>1.6</v>
+          </cell>
+          <cell r="Y76">
+            <v>12.1</v>
+          </cell>
+          <cell r="Z76">
+            <v>12.1</v>
+          </cell>
+        </row>
+        <row r="77">
+          <cell r="C77" t="str">
+            <v>Heat storage discharger</v>
+          </cell>
+          <cell r="S77">
+            <v>1</v>
+          </cell>
+        </row>
+        <row r="78">
+          <cell r="C78" t="str">
+            <v>Heat storage charger</v>
+          </cell>
+          <cell r="S78">
+            <v>1</v>
+          </cell>
+        </row>
+        <row r="79">
+          <cell r="C79" t="str">
+            <v>Large heat storage discharger</v>
+          </cell>
+          <cell r="S79">
+            <v>1.5</v>
+          </cell>
+        </row>
+        <row r="80">
+          <cell r="C80" t="str">
+            <v>Large heat storage charger</v>
+          </cell>
+          <cell r="S80">
+            <v>1.5</v>
+          </cell>
+        </row>
+        <row r="81">
+          <cell r="C81" t="str">
+            <v>Seasonal heat storage discharger</v>
+          </cell>
+          <cell r="S81">
+            <v>2</v>
+          </cell>
+        </row>
+        <row r="82">
+          <cell r="C82" t="str">
+            <v>Seasonal heat storage charger</v>
+          </cell>
+          <cell r="S82">
+            <v>2</v>
+          </cell>
+        </row>
+        <row r="84">
+          <cell r="C84" t="str">
+            <v>DR upwards 2</v>
+          </cell>
+        </row>
+        <row r="85">
+          <cell r="C85" t="str">
+            <v>DR upwards 1</v>
+          </cell>
+        </row>
+        <row r="86">
+          <cell r="C86" t="str">
+            <v>DR cutoff tier 3</v>
+          </cell>
+          <cell r="S86">
+            <v>2000</v>
+          </cell>
+        </row>
+        <row r="87">
+          <cell r="C87" t="str">
+            <v>DR cutoff tier 2</v>
+          </cell>
+          <cell r="S87">
+            <v>1000</v>
+          </cell>
+        </row>
+        <row r="88">
+          <cell r="C88" t="str">
+            <v>DR cutoff tier 1</v>
+          </cell>
+          <cell r="S88">
+            <v>400</v>
+          </cell>
+        </row>
+        <row r="90">
+          <cell r="C90" t="str">
+            <v>Electrolyser</v>
+          </cell>
+          <cell r="S90">
+            <v>1</v>
+          </cell>
+          <cell r="Y90">
+            <v>15</v>
+          </cell>
+          <cell r="Z90">
+            <v>15</v>
+          </cell>
+        </row>
+        <row r="91">
+          <cell r="C91" t="str">
+            <v>Electrolyser-SOEC</v>
+          </cell>
+          <cell r="S91">
+            <v>1</v>
+          </cell>
+          <cell r="Y91">
+            <v>25</v>
+          </cell>
+          <cell r="Z91">
+            <v>25</v>
+          </cell>
+        </row>
+        <row r="92">
+          <cell r="C92" t="str">
+            <v>Hydrogen OCGT</v>
+          </cell>
+          <cell r="S92">
+            <v>5</v>
+          </cell>
+          <cell r="Y92">
+            <v>30</v>
+          </cell>
+        </row>
+        <row r="93">
+          <cell r="C93" t="str">
+            <v>Short-term hydrogen storage discharger</v>
+          </cell>
+          <cell r="S93">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="94">
+          <cell r="C94" t="str">
+            <v>Short-term hydrogen storage charger</v>
+          </cell>
+          <cell r="S94">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="95">
+          <cell r="C95" t="str">
+            <v>Long-term hydrogen storage discharger</v>
+          </cell>
+          <cell r="S95">
+            <v>0</v>
+          </cell>
+          <cell r="Y95">
+            <v>0</v>
+          </cell>
+        </row>
+        <row r="96">
+          <cell r="C96" t="str">
+            <v>Long-term hydrogen storage charger</v>
+          </cell>
+          <cell r="S96">
+            <v>1</v>
+          </cell>
+          <cell r="Y96">
+            <v>0</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4E105637-66C0-4B67-968B-A8C9BC84D774}" name="Table2" displayName="Table2" ref="A1:J41" totalsRowShown="0" headerRowDxfId="9">
   <autoFilter ref="A1:J41" xr:uid="{4E105637-66C0-4B67-968B-A8C9BC84D774}"/>
@@ -677,12 +2148,12 @@
     <tableColumn id="2" xr3:uid="{9F2751A6-04EC-4ED2-AB42-B8EA5F26204C}" name="Grid"/>
     <tableColumn id="4" xr3:uid="{9BB2F988-4BF3-43BE-825B-61D7ED214C20}" name="Scenario" dataDxfId="7"/>
     <tableColumn id="5" xr3:uid="{B2E82F1D-6AE0-4465-8201-B09B1A163DBC}" name="Year" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{A3BED5EB-08A7-4F3F-AB5F-17A0A75BE225}" name="nodeBalance" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{70FFAE63-9B59-49B3-A41F-076293B979F8}" name="upwardLimit" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{E4BBBCCD-F5BD-4D0B-9262-F84C87E3CCE6}" name="reference" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{F7666183-1180-4234-AD88-B1F9E55F6267}" name="balancePenalty" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{84FDFFC6-278E-4FC6-9D54-9736721D6070}" name="maxSpill" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{4277BD29-04AE-4F26-8CE8-222C6FFCB3F8}" name="Method" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{A3BED5EB-08A7-4F3F-AB5F-17A0A75BE225}" name="nodeBalance" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{70FFAE63-9B59-49B3-A41F-076293B979F8}" name="upwardLimit" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{E4BBBCCD-F5BD-4D0B-9262-F84C87E3CCE6}" name="reference" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{F7666183-1180-4234-AD88-B1F9E55F6267}" name="balancePenalty" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{84FDFFC6-278E-4FC6-9D54-9736721D6070}" name="maxSpill" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{4277BD29-04AE-4F26-8CE8-222C6FFCB3F8}" name="Method" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -965,6 +2436,7 @@
     <col min="7" max="7" width="12" style="13" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.28515625" style="13" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2106,7 +3578,7 @@
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:U59"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
@@ -2114,11 +3586,14 @@
     <col min="3" max="3" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>25</v>
       </c>
@@ -2134,14 +3609,23 @@
       <c r="E1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="30" t="s">
+        <v>102</v>
+      </c>
+      <c r="G1" s="30" t="s">
+        <v>110</v>
+      </c>
+      <c r="H1" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="I1" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2157,8 +3641,20 @@
       <c r="E2" s="1">
         <v>5782</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F2">
+        <f>ROUND(SUMIFS(R$31:R$36,$Q$31:$Q$36,$B2) * (1 + SUMIFS($U$7:$U$28,$Q$7:$Q$28,$A2)), 2)</f>
+        <v>2.48</v>
+      </c>
+      <c r="G2">
+        <f t="shared" ref="G2:H2" si="0">ROUND(SUMIFS(S$31:S$36,$Q$31:$Q$36,$B2) * (1 + SUMIFS($U$7:$U$28,$Q$7:$Q$28,$A2)), 2)</f>
+        <v>6.2</v>
+      </c>
+      <c r="H2">
+        <f t="shared" si="0"/>
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -2174,8 +3670,20 @@
       <c r="E3" s="1">
         <v>113.94</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F3">
+        <f t="shared" ref="F3:F59" si="1">ROUND(SUMIFS(R$31:R$36,$Q$31:$Q$36,$B3) * (1 + SUMIFS($U$7:$U$28,$Q$7:$Q$28,$A3)), 2)</f>
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G59" si="2">ROUND(SUMIFS(S$31:S$36,$Q$31:$Q$36,$B3) * (1 + SUMIFS($U$7:$U$28,$Q$7:$Q$28,$A3)), 2)</f>
+        <v>6.17</v>
+      </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H59" si="3">ROUND(SUMIFS(T$31:T$36,$Q$31:$Q$36,$B3) * (1 + SUMIFS($U$7:$U$28,$Q$7:$Q$28,$A3)), 2)</f>
+        <v>6.17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2191,8 +3699,20 @@
       <c r="E4" s="1">
         <v>4031</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F4">
+        <f t="shared" si="1"/>
+        <v>3.2</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="2"/>
+        <v>8.01</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="3"/>
+        <v>8.01</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2208,8 +3728,20 @@
       <c r="E5" s="1">
         <v>4036</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>2.44</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="2"/>
+        <v>6.09</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="3"/>
+        <v>6.09</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -2225,8 +3757,32 @@
       <c r="E6" s="1">
         <v>3300</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>2.02</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="2"/>
+        <v>5.04</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="3"/>
+        <v>5.04</v>
+      </c>
+      <c r="R6" t="s">
+        <v>103</v>
+      </c>
+      <c r="S6" t="s">
+        <v>104</v>
+      </c>
+      <c r="T6" t="s">
+        <v>105</v>
+      </c>
+      <c r="U6" s="27" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -2242,8 +3798,39 @@
       <c r="E7" s="1">
         <v>20500</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>2.3199999999999998</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="2"/>
+        <v>5.8</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="3"/>
+        <v>5.8</v>
+      </c>
+      <c r="Q7" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="R7" s="6">
+        <f>'[1]vomcost mult'!O11</f>
+        <v>45140</v>
+      </c>
+      <c r="S7" s="28">
+        <f>'[1]vomcost mult'!P11</f>
+        <v>0.12757648618174755</v>
+      </c>
+      <c r="T7" s="6">
+        <f>'[1]vomcost mult'!Q11</f>
+        <v>1</v>
+      </c>
+      <c r="U7" s="29">
+        <f>'[1]vomcost mult'!R11</f>
+        <v>0.128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -2259,8 +3846,39 @@
       <c r="E8" s="1">
         <v>128</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F8">
+        <f t="shared" si="1"/>
+        <v>1.69</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="2"/>
+        <v>4.22</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="3"/>
+        <v>4.22</v>
+      </c>
+      <c r="Q8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="R8" s="6">
+        <f>'[1]vomcost mult'!O12</f>
+        <v>44440</v>
+      </c>
+      <c r="S8" s="28">
+        <f>'[1]vomcost mult'!P12</f>
+        <v>0.12078898170883434</v>
+      </c>
+      <c r="T8" s="6">
+        <f>'[1]vomcost mult'!Q12</f>
+        <v>1</v>
+      </c>
+      <c r="U8" s="29">
+        <f>'[1]vomcost mult'!R12</f>
+        <v>0.121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -2276,8 +3894,39 @@
       <c r="E9" s="1">
         <v>1557</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F9">
+        <f t="shared" si="1"/>
+        <v>1.54</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="2"/>
+        <v>3.86</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="3"/>
+        <v>3.86</v>
+      </c>
+      <c r="Q9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="R9" s="6">
+        <f>'[1]vomcost mult'!O13</f>
+        <v>96081</v>
+      </c>
+      <c r="S9" s="28">
+        <f>'[1]vomcost mult'!P13</f>
+        <v>0.4556524459454061</v>
+      </c>
+      <c r="T9" s="6">
+        <f>'[1]vomcost mult'!Q13</f>
+        <v>1</v>
+      </c>
+      <c r="U9" s="29">
+        <f>'[1]vomcost mult'!R13</f>
+        <v>0.45600000000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -2293,8 +3942,39 @@
       <c r="E10" s="1">
         <v>38</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F10">
+        <f t="shared" si="1"/>
+        <v>2.6</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="2"/>
+        <v>6.49</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="3"/>
+        <v>6.49</v>
+      </c>
+      <c r="Q10" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="R10" s="6">
+        <f>'[1]vomcost mult'!O14</f>
+        <v>43110</v>
+      </c>
+      <c r="S10" s="28">
+        <f>'[1]vomcost mult'!P14</f>
+        <v>0.1075929542938924</v>
+      </c>
+      <c r="T10" s="6">
+        <f>'[1]vomcost mult'!Q14</f>
+        <v>1</v>
+      </c>
+      <c r="U10" s="29">
+        <f>'[1]vomcost mult'!R14</f>
+        <v>0.108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -2310,8 +3990,39 @@
       <c r="E11" s="1">
         <v>506.5</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F11">
+        <f t="shared" si="1"/>
+        <v>1.52</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="2"/>
+        <v>3.8</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="3"/>
+        <v>3.8</v>
+      </c>
+      <c r="Q11" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="R11" s="6">
+        <f>'[1]vomcost mult'!O15</f>
+        <v>58160</v>
+      </c>
+      <c r="S11" s="28">
+        <f>'[1]vomcost mult'!P15</f>
+        <v>0.2376393292909858</v>
+      </c>
+      <c r="T11" s="6">
+        <f>'[1]vomcost mult'!Q15</f>
+        <v>1.05</v>
+      </c>
+      <c r="U11" s="29">
+        <f>'[1]vomcost mult'!R15</f>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -2327,8 +4038,39 @@
       <c r="E12" s="1">
         <v>1826</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F12">
+        <f t="shared" si="1"/>
+        <v>2.56</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="2"/>
+        <v>6.41</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="3"/>
+        <v>6.41</v>
+      </c>
+      <c r="Q12" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="R12" s="6">
+        <f>'[1]vomcost mult'!O16</f>
+        <v>58160</v>
+      </c>
+      <c r="S12" s="28">
+        <f>'[1]vomcost mult'!P16</f>
+        <v>0.2376393292909858</v>
+      </c>
+      <c r="T12" s="6">
+        <f>'[1]vomcost mult'!Q16</f>
+        <v>1</v>
+      </c>
+      <c r="U12" s="29">
+        <f>'[1]vomcost mult'!R16</f>
+        <v>0.23799999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -2344,8 +4086,39 @@
       <c r="E13" s="2">
         <v>2429.5540000000001</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="2"/>
+        <v>5.64</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="3"/>
+        <v>5.64</v>
+      </c>
+      <c r="Q13" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="R13" s="6">
+        <f>'[1]vomcost mult'!O17</f>
+        <v>21060</v>
+      </c>
+      <c r="S13" s="28">
+        <f>'[1]vomcost mult'!P17</f>
+        <v>-0.20352670171052795</v>
+      </c>
+      <c r="T13" s="6">
+        <f>'[1]vomcost mult'!Q17</f>
+        <v>1</v>
+      </c>
+      <c r="U13" s="29">
+        <f>'[1]vomcost mult'!R17</f>
+        <v>-0.20399999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -2361,8 +4134,39 @@
       <c r="E14" s="2">
         <v>8152</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>2.91</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="2"/>
+        <v>7.28</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="3"/>
+        <v>7.28</v>
+      </c>
+      <c r="Q14" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="R14" s="6">
+        <f>'[1]vomcost mult'!O18</f>
+        <v>27800</v>
+      </c>
+      <c r="S14" s="28">
+        <f>'[1]vomcost mult'!P18</f>
+        <v>-8.2940272641919402E-2</v>
+      </c>
+      <c r="T14" s="6">
+        <f>'[1]vomcost mult'!Q18</f>
+        <v>1</v>
+      </c>
+      <c r="U14" s="29">
+        <f>'[1]vomcost mult'!R18</f>
+        <v>-8.3000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -2378,8 +4182,39 @@
       <c r="E15" s="2">
         <v>1297</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F15">
+        <f t="shared" si="1"/>
+        <v>2.2200000000000002</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="2"/>
+        <v>5.54</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="3"/>
+        <v>5.54</v>
+      </c>
+      <c r="Q15" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="R15" s="6">
+        <f>'[1]vomcost mult'!O19</f>
+        <v>43110</v>
+      </c>
+      <c r="S15" s="28">
+        <f>'[1]vomcost mult'!P19</f>
+        <v>0.1075929542938924</v>
+      </c>
+      <c r="T15" s="6">
+        <f>'[1]vomcost mult'!Q19</f>
+        <v>1</v>
+      </c>
+      <c r="U15" s="29">
+        <f>'[1]vomcost mult'!R19</f>
+        <v>0.108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>10</v>
       </c>
@@ -2395,8 +4230,39 @@
       <c r="E16" s="2">
         <v>10970</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F16">
+        <f t="shared" si="1"/>
+        <v>1.83</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="2"/>
+        <v>4.59</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="3"/>
+        <v>4.59</v>
+      </c>
+      <c r="Q16" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="R16" s="6">
+        <f>'[1]vomcost mult'!O20</f>
+        <v>38110</v>
+      </c>
+      <c r="S16" s="28">
+        <f>'[1]vomcost mult'!P20</f>
+        <v>5.4053880212171543E-2</v>
+      </c>
+      <c r="T16" s="6">
+        <f>'[1]vomcost mult'!Q20</f>
+        <v>1</v>
+      </c>
+      <c r="U16" s="29">
+        <f>'[1]vomcost mult'!R20</f>
+        <v>5.3999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -2412,8 +4278,39 @@
       <c r="E17" s="2">
         <v>3200</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F17">
+        <f t="shared" si="1"/>
+        <v>2.2200000000000002</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="2"/>
+        <v>5.54</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="3"/>
+        <v>5.54</v>
+      </c>
+      <c r="Q17" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="R17" s="6">
+        <f>'[1]vomcost mult'!O21</f>
+        <v>19690</v>
+      </c>
+      <c r="S17" s="28">
+        <f>'[1]vomcost mult'!P21</f>
+        <v>-0.2327393524218774</v>
+      </c>
+      <c r="T17" s="6">
+        <f>'[1]vomcost mult'!Q21</f>
+        <v>1</v>
+      </c>
+      <c r="U17" s="29">
+        <f>'[1]vomcost mult'!R21</f>
+        <v>-0.23300000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>12</v>
       </c>
@@ -2429,8 +4326,39 @@
       <c r="E18" s="2">
         <v>8477</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F18">
+        <f t="shared" si="1"/>
+        <v>2.11</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="2"/>
+        <v>5.27</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="3"/>
+        <v>5.27</v>
+      </c>
+      <c r="Q18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="R18" s="6">
+        <f>'[1]vomcost mult'!O22</f>
+        <v>16910</v>
+      </c>
+      <c r="S18" s="28">
+        <f>'[1]vomcost mult'!P22</f>
+        <v>-0.29884146096225389</v>
+      </c>
+      <c r="T18" s="6">
+        <f>'[1]vomcost mult'!Q22</f>
+        <v>1</v>
+      </c>
+      <c r="U18" s="29">
+        <f>'[1]vomcost mult'!R22</f>
+        <v>-0.29899999999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -2446,8 +4374,39 @@
       <c r="E19" s="2">
         <v>183.8</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F19">
+        <f t="shared" si="1"/>
+        <v>1.38</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="2"/>
+        <v>3.45</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="3"/>
+        <v>3.45</v>
+      </c>
+      <c r="Q19" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="R19" s="6">
+        <f>'[1]vomcost mult'!O23</f>
+        <v>50880</v>
+      </c>
+      <c r="S19" s="28">
+        <f>'[1]vomcost mult'!P23</f>
+        <v>0.17956203408036178</v>
+      </c>
+      <c r="T19" s="6">
+        <f>'[1]vomcost mult'!Q23</f>
+        <v>1</v>
+      </c>
+      <c r="U19" s="29">
+        <f>'[1]vomcost mult'!R23</f>
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -2463,8 +4422,39 @@
       <c r="E20" s="2">
         <v>5315</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F20">
+        <f t="shared" si="1"/>
+        <v>2.36</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="2"/>
+        <v>5.91</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="3"/>
+        <v>5.91</v>
+      </c>
+      <c r="Q20" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="R20" s="6">
+        <f>'[1]vomcost mult'!O24</f>
+        <v>66460</v>
+      </c>
+      <c r="S20" s="28">
+        <f>'[1]vomcost mult'!P24</f>
+        <v>0.2955752683826966</v>
+      </c>
+      <c r="T20" s="6">
+        <f>'[1]vomcost mult'!Q24</f>
+        <v>1.05</v>
+      </c>
+      <c r="U20" s="29">
+        <f>'[1]vomcost mult'!R24</f>
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -2480,8 +4470,39 @@
       <c r="E21" s="2">
         <v>8055</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F21">
+        <f t="shared" si="1"/>
+        <v>2.35</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="2"/>
+        <v>5.87</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="3"/>
+        <v>5.87</v>
+      </c>
+      <c r="Q21" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="R21" s="6">
+        <f>'[1]vomcost mult'!O25</f>
+        <v>66460</v>
+      </c>
+      <c r="S21" s="28">
+        <f>'[1]vomcost mult'!P25</f>
+        <v>0.2955752683826966</v>
+      </c>
+      <c r="T21" s="6">
+        <f>'[1]vomcost mult'!Q25</f>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="U21" s="29">
+        <f>'[1]vomcost mult'!R25</f>
+        <v>0.32500000000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -2497,8 +4518,39 @@
       <c r="E22" s="2">
         <v>2331</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F22">
+        <f t="shared" si="1"/>
+        <v>2.33</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="2"/>
+        <v>5.83</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="3"/>
+        <v>5.83</v>
+      </c>
+      <c r="Q22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="R22" s="6">
+        <f>'[1]vomcost mult'!O26</f>
+        <v>66460</v>
+      </c>
+      <c r="S22" s="28">
+        <f>'[1]vomcost mult'!P26</f>
+        <v>0.2955752683826966</v>
+      </c>
+      <c r="T22" s="6">
+        <f>'[1]vomcost mult'!Q26</f>
+        <v>1</v>
+      </c>
+      <c r="U22" s="29">
+        <f>'[1]vomcost mult'!R26</f>
+        <v>0.29599999999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -2514,8 +4566,39 @@
       <c r="E23" s="2">
         <v>237</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F23">
+        <f t="shared" si="1"/>
+        <v>2.31</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="2"/>
+        <v>5.79</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="3"/>
+        <v>5.79</v>
+      </c>
+      <c r="Q23" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="R23" s="6">
+        <f>'[1]vomcost mult'!O27</f>
+        <v>16470</v>
+      </c>
+      <c r="S23" s="28">
+        <f>'[1]vomcost mult'!P27</f>
+        <v>-0.31029146939024133</v>
+      </c>
+      <c r="T23" s="6">
+        <f>'[1]vomcost mult'!Q27</f>
+        <v>1</v>
+      </c>
+      <c r="U23" s="29">
+        <f>'[1]vomcost mult'!R27</f>
+        <v>-0.31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>0</v>
       </c>
@@ -2531,8 +4614,39 @@
       <c r="E24" s="3">
         <v>3459.28</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F24">
+        <f t="shared" si="1"/>
+        <v>1.69</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="2"/>
+        <v>4.51</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="3"/>
+        <v>4.51</v>
+      </c>
+      <c r="Q24" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="R24" s="6">
+        <f>'[1]vomcost mult'!O28</f>
+        <v>48310</v>
+      </c>
+      <c r="S24" s="28">
+        <f>'[1]vomcost mult'!P28</f>
+        <v>0.15705196892652412</v>
+      </c>
+      <c r="T24" s="6">
+        <f>'[1]vomcost mult'!Q28</f>
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="U24" s="29">
+        <f>'[1]vomcost mult'!R28</f>
+        <v>0.18099999999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>8</v>
       </c>
@@ -2545,11 +4659,42 @@
       <c r="D25">
         <v>1</v>
       </c>
-      <c r="G25" t="s">
+      <c r="F25">
+        <f t="shared" si="1"/>
+        <v>2.1800000000000002</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="2"/>
+        <v>5.82</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="3"/>
+        <v>5.82</v>
+      </c>
+      <c r="J25" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="Q25" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="R25" s="6">
+        <f>'[1]vomcost mult'!O29</f>
+        <v>48310</v>
+      </c>
+      <c r="S25" s="28">
+        <f>'[1]vomcost mult'!P29</f>
+        <v>0.15705196892652412</v>
+      </c>
+      <c r="T25" s="6">
+        <f>'[1]vomcost mult'!Q29</f>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="U25" s="29">
+        <f>'[1]vomcost mult'!R29</f>
+        <v>0.17299999999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>9</v>
       </c>
@@ -2565,8 +4710,39 @@
       <c r="E26" s="3">
         <v>1644</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F26">
+        <f t="shared" si="1"/>
+        <v>1.66</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="2"/>
+        <v>4.43</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="3"/>
+        <v>4.43</v>
+      </c>
+      <c r="Q26" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="R26" s="6">
+        <f>'[1]vomcost mult'!O30</f>
+        <v>48310</v>
+      </c>
+      <c r="S26" s="28">
+        <f>'[1]vomcost mult'!P30</f>
+        <v>0.15705196892652412</v>
+      </c>
+      <c r="T26" s="6">
+        <f>'[1]vomcost mult'!Q30</f>
+        <v>1.05</v>
+      </c>
+      <c r="U26" s="29">
+        <f>'[1]vomcost mult'!R30</f>
+        <v>0.16500000000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>10</v>
       </c>
@@ -2582,8 +4758,39 @@
       <c r="E27" s="3">
         <v>2683</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F27">
+        <f t="shared" si="1"/>
+        <v>1.38</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="2"/>
+        <v>3.67</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="3"/>
+        <v>3.67</v>
+      </c>
+      <c r="Q27" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="R27" s="6">
+        <f>'[1]vomcost mult'!O31</f>
+        <v>48310</v>
+      </c>
+      <c r="S27" s="28">
+        <f>'[1]vomcost mult'!P31</f>
+        <v>0.15705196892652412</v>
+      </c>
+      <c r="T27" s="6">
+        <f>'[1]vomcost mult'!Q31</f>
+        <v>1</v>
+      </c>
+      <c r="U27" s="29">
+        <f>'[1]vomcost mult'!R31</f>
+        <v>0.157</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -2599,8 +4806,39 @@
       <c r="E28" s="3">
         <v>1850</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F28">
+        <f t="shared" si="1"/>
+        <v>1.58</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="2"/>
+        <v>4.22</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="3"/>
+        <v>4.22</v>
+      </c>
+      <c r="Q28" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="R28" s="6">
+        <f>'[1]vomcost mult'!O32</f>
+        <v>49193</v>
+      </c>
+      <c r="S28" s="28">
+        <f>'[1]vomcost mult'!P32</f>
+        <v>0.16491823994601576</v>
+      </c>
+      <c r="T28" s="6">
+        <f>'[1]vomcost mult'!Q32</f>
+        <v>1</v>
+      </c>
+      <c r="U28" s="29">
+        <f>'[1]vomcost mult'!R32</f>
+        <v>0.16500000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>16</v>
       </c>
@@ -2616,8 +4854,20 @@
       <c r="E29" s="3">
         <v>4631.3999999999996</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F29">
+        <f t="shared" si="1"/>
+        <v>1.97</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="2"/>
+        <v>5.24</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="3"/>
+        <v>5.24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>17</v>
       </c>
@@ -2633,8 +4883,29 @@
       <c r="E30" s="3">
         <v>5540.4</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F30">
+        <f t="shared" si="1"/>
+        <v>1.99</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="2"/>
+        <v>5.3</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="3"/>
+        <v>5.3</v>
+      </c>
+      <c r="R30" t="s">
+        <v>102</v>
+      </c>
+      <c r="S30" t="s">
+        <v>110</v>
+      </c>
+      <c r="T30" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>18</v>
       </c>
@@ -2650,8 +4921,35 @@
       <c r="E31" s="3">
         <v>23605.1</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F31">
+        <f t="shared" si="1"/>
+        <v>1.94</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="2"/>
+        <v>5.18</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="3"/>
+        <v>5.18</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>6</v>
+      </c>
+      <c r="R31">
+        <f>SUMIFS([2]unittypedata!$S:$S,[2]unittypedata!$C:$C, $Q31)</f>
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="S31">
+        <f>SUMIFS([2]unittypedata!$Y:$Y,[2]unittypedata!$C:$C, $Q31)</f>
+        <v>5.5</v>
+      </c>
+      <c r="T31">
+        <f>SUMIFS([2]unittypedata!$Z:$Z,[2]unittypedata!$C:$C, $Q31)</f>
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>19</v>
       </c>
@@ -2667,8 +4965,35 @@
       <c r="E32" s="3">
         <v>178.8</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F32">
+        <f t="shared" si="1"/>
+        <v>1.04</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="2"/>
+        <v>2.76</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="3"/>
+        <v>2.76</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>5</v>
+      </c>
+      <c r="R32">
+        <f>SUMIFS([2]unittypedata!$S:$S,[2]unittypedata!$C:$C, $Q32)</f>
+        <v>2</v>
+      </c>
+      <c r="S32">
+        <f>SUMIFS([2]unittypedata!$Y:$Y,[2]unittypedata!$C:$C, $Q32)</f>
+        <v>5</v>
+      </c>
+      <c r="T32">
+        <f>SUMIFS([2]unittypedata!$Z:$Z,[2]unittypedata!$C:$C, $Q32)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>0</v>
       </c>
@@ -2684,8 +5009,35 @@
       <c r="E33" s="8">
         <v>2560</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F33">
+        <f t="shared" si="1"/>
+        <v>1.58</v>
+      </c>
+      <c r="G33">
+        <f t="shared" si="2"/>
+        <v>3.95</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="3"/>
+        <v>3.95</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>4</v>
+      </c>
+      <c r="R33">
+        <f>SUMIFS([2]unittypedata!$S:$S,[2]unittypedata!$C:$C, $Q33)</f>
+        <v>1.5</v>
+      </c>
+      <c r="S33">
+        <f>SUMIFS([2]unittypedata!$Y:$Y,[2]unittypedata!$C:$C, $Q33)</f>
+        <v>4</v>
+      </c>
+      <c r="T33">
+        <f>SUMIFS([2]unittypedata!$Z:$Z,[2]unittypedata!$C:$C, $Q33)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>8</v>
       </c>
@@ -2698,11 +5050,38 @@
       <c r="D34">
         <v>1</v>
       </c>
-      <c r="G34" t="s">
+      <c r="F34">
+        <f t="shared" si="1"/>
+        <v>2.04</v>
+      </c>
+      <c r="G34">
+        <f t="shared" si="2"/>
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="H34">
+        <f t="shared" si="3"/>
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="J34" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="Q34" t="s">
+        <v>3</v>
+      </c>
+      <c r="R34">
+        <f>SUMIFS([2]unittypedata!$S:$S,[2]unittypedata!$C:$C, $Q34)</f>
+        <v>1.4</v>
+      </c>
+      <c r="S34">
+        <f>SUMIFS([2]unittypedata!$Y:$Y,[2]unittypedata!$C:$C, $Q34)</f>
+        <v>3.5</v>
+      </c>
+      <c r="T34">
+        <f>SUMIFS([2]unittypedata!$Z:$Z,[2]unittypedata!$C:$C, $Q34)</f>
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>9</v>
       </c>
@@ -2718,8 +5097,35 @@
       <c r="E35" s="8">
         <v>1361</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F35">
+        <f t="shared" si="1"/>
+        <v>1.55</v>
+      </c>
+      <c r="G35">
+        <f t="shared" si="2"/>
+        <v>3.88</v>
+      </c>
+      <c r="H35">
+        <f t="shared" si="3"/>
+        <v>3.88</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>2</v>
+      </c>
+      <c r="R35">
+        <f>SUMIFS([2]unittypedata!$S:$S,[2]unittypedata!$C:$C, $Q35)</f>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="S35">
+        <f>SUMIFS([2]unittypedata!$Y:$Y,[2]unittypedata!$C:$C, $Q35)</f>
+        <v>3.1</v>
+      </c>
+      <c r="T35">
+        <f>SUMIFS([2]unittypedata!$Z:$Z,[2]unittypedata!$C:$C, $Q35)</f>
+        <v>3.1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>10</v>
       </c>
@@ -2735,8 +5141,35 @@
       <c r="E36" s="8">
         <v>2424</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F36">
+        <f t="shared" si="1"/>
+        <v>1.28</v>
+      </c>
+      <c r="G36">
+        <f t="shared" si="2"/>
+        <v>3.21</v>
+      </c>
+      <c r="H36">
+        <f t="shared" si="3"/>
+        <v>3.21</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>1</v>
+      </c>
+      <c r="R36">
+        <f>SUMIFS([2]unittypedata!$S:$S,[2]unittypedata!$C:$C, $Q36)</f>
+        <v>1</v>
+      </c>
+      <c r="S36">
+        <f>SUMIFS([2]unittypedata!$Y:$Y,[2]unittypedata!$C:$C, $Q36)</f>
+        <v>3</v>
+      </c>
+      <c r="T36">
+        <f>SUMIFS([2]unittypedata!$Z:$Z,[2]unittypedata!$C:$C, $Q36)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -2752,8 +5185,20 @@
       <c r="E37" s="8">
         <v>1850</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F37">
+        <f t="shared" si="1"/>
+        <v>1.48</v>
+      </c>
+      <c r="G37">
+        <f t="shared" si="2"/>
+        <v>3.69</v>
+      </c>
+      <c r="H37">
+        <f t="shared" si="3"/>
+        <v>3.69</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>16</v>
       </c>
@@ -2769,8 +5214,20 @@
       <c r="E38" s="8">
         <v>84</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F38">
+        <f t="shared" si="1"/>
+        <v>1.83</v>
+      </c>
+      <c r="G38">
+        <f t="shared" si="2"/>
+        <v>4.59</v>
+      </c>
+      <c r="H38">
+        <f t="shared" si="3"/>
+        <v>4.59</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>17</v>
       </c>
@@ -2783,11 +5240,23 @@
       <c r="D39">
         <v>1</v>
       </c>
-      <c r="G39" t="s">
+      <c r="F39">
+        <f t="shared" si="1"/>
+        <v>1.86</v>
+      </c>
+      <c r="G39">
+        <f t="shared" si="2"/>
+        <v>4.6399999999999997</v>
+      </c>
+      <c r="H39">
+        <f t="shared" si="3"/>
+        <v>4.6399999999999997</v>
+      </c>
+      <c r="J39" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>18</v>
       </c>
@@ -2803,8 +5272,20 @@
       <c r="E40" s="8">
         <v>1030</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F40">
+        <f t="shared" si="1"/>
+        <v>1.81</v>
+      </c>
+      <c r="G40">
+        <f t="shared" si="2"/>
+        <v>4.54</v>
+      </c>
+      <c r="H40">
+        <f t="shared" si="3"/>
+        <v>4.54</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>19</v>
       </c>
@@ -2820,8 +5301,20 @@
       <c r="E41" s="8">
         <v>172</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F41">
+        <f t="shared" si="1"/>
+        <v>0.97</v>
+      </c>
+      <c r="G41">
+        <f t="shared" si="2"/>
+        <v>2.42</v>
+      </c>
+      <c r="H41">
+        <f t="shared" si="3"/>
+        <v>2.42</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>0</v>
       </c>
@@ -2834,11 +5327,23 @@
       <c r="D42">
         <v>1</v>
       </c>
-      <c r="G42" t="s">
+      <c r="F42">
+        <f t="shared" si="1"/>
+        <v>1.24</v>
+      </c>
+      <c r="G42">
+        <f t="shared" si="2"/>
+        <v>3.5</v>
+      </c>
+      <c r="H42">
+        <f t="shared" si="3"/>
+        <v>3.5</v>
+      </c>
+      <c r="J42" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>7</v>
       </c>
@@ -2854,8 +5359,20 @@
       <c r="E43" s="7">
         <v>1308</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F43">
+        <f t="shared" si="1"/>
+        <v>1.23</v>
+      </c>
+      <c r="G43">
+        <f t="shared" si="2"/>
+        <v>3.48</v>
+      </c>
+      <c r="H43">
+        <f t="shared" si="3"/>
+        <v>3.48</v>
+      </c>
+    </row>
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>8</v>
       </c>
@@ -2871,8 +5388,20 @@
       <c r="E44" s="7">
         <v>3989</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F44">
+        <f t="shared" si="1"/>
+        <v>1.6</v>
+      </c>
+      <c r="G44">
+        <f t="shared" si="2"/>
+        <v>4.51</v>
+      </c>
+      <c r="H44">
+        <f t="shared" si="3"/>
+        <v>4.51</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>9</v>
       </c>
@@ -2888,8 +5417,20 @@
       <c r="E45" s="7">
         <v>6056</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F45">
+        <f t="shared" si="1"/>
+        <v>1.22</v>
+      </c>
+      <c r="G45">
+        <f t="shared" si="2"/>
+        <v>3.43</v>
+      </c>
+      <c r="H45">
+        <f t="shared" si="3"/>
+        <v>3.43</v>
+      </c>
+    </row>
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>10</v>
       </c>
@@ -2905,8 +5446,20 @@
       <c r="E46" s="7">
         <v>3330</v>
       </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F46">
+        <f t="shared" si="1"/>
+        <v>1.01</v>
+      </c>
+      <c r="G46">
+        <f t="shared" si="2"/>
+        <v>2.84</v>
+      </c>
+      <c r="H46">
+        <f t="shared" si="3"/>
+        <v>2.84</v>
+      </c>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>12</v>
       </c>
@@ -2922,8 +5475,20 @@
       <c r="E47" s="7">
         <v>1950</v>
       </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F47">
+        <f t="shared" si="1"/>
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="G47">
+        <f t="shared" si="2"/>
+        <v>3.27</v>
+      </c>
+      <c r="H47">
+        <f t="shared" si="3"/>
+        <v>3.27</v>
+      </c>
+    </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>13</v>
       </c>
@@ -2939,8 +5504,20 @@
       <c r="E48" s="7">
         <v>900</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F48">
+        <f t="shared" si="1"/>
+        <v>0.84</v>
+      </c>
+      <c r="G48">
+        <f t="shared" si="2"/>
+        <v>2.38</v>
+      </c>
+      <c r="H48">
+        <f t="shared" si="3"/>
+        <v>2.38</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>19</v>
       </c>
@@ -2956,8 +5533,20 @@
       <c r="E49" s="7">
         <v>1323</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F49">
+        <f t="shared" si="1"/>
+        <v>0.76</v>
+      </c>
+      <c r="G49">
+        <f t="shared" si="2"/>
+        <v>2.14</v>
+      </c>
+      <c r="H49">
+        <f t="shared" si="3"/>
+        <v>2.14</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>24</v>
       </c>
@@ -2973,8 +5562,20 @@
       <c r="E50" s="7">
         <v>2744</v>
       </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F50">
+        <f t="shared" si="1"/>
+        <v>1.28</v>
+      </c>
+      <c r="G50">
+        <f t="shared" si="2"/>
+        <v>3.61</v>
+      </c>
+      <c r="H50">
+        <f t="shared" si="3"/>
+        <v>3.61</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>0</v>
       </c>
@@ -2987,11 +5588,23 @@
       <c r="D51">
         <v>1</v>
       </c>
-      <c r="G51" t="s">
+      <c r="F51">
+        <f t="shared" si="1"/>
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="G51">
+        <f t="shared" si="2"/>
+        <v>3.38</v>
+      </c>
+      <c r="H51">
+        <f t="shared" si="3"/>
+        <v>3.38</v>
+      </c>
+      <c r="J51" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>7</v>
       </c>
@@ -3007,8 +5620,20 @@
       <c r="E52" s="18">
         <v>1150</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F52">
+        <f t="shared" si="1"/>
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="G52">
+        <f t="shared" si="2"/>
+        <v>3.36</v>
+      </c>
+      <c r="H52">
+        <f t="shared" si="3"/>
+        <v>3.36</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>8</v>
       </c>
@@ -3024,8 +5649,20 @@
       <c r="E53" s="18">
         <v>3938</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F53">
+        <f t="shared" si="1"/>
+        <v>1.46</v>
+      </c>
+      <c r="G53">
+        <f t="shared" si="2"/>
+        <v>4.37</v>
+      </c>
+      <c r="H53">
+        <f t="shared" si="3"/>
+        <v>4.37</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>9</v>
       </c>
@@ -3041,8 +5678,20 @@
       <c r="E54" s="18">
         <v>6068</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F54">
+        <f t="shared" si="1"/>
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="G54">
+        <f t="shared" si="2"/>
+        <v>3.32</v>
+      </c>
+      <c r="H54">
+        <f t="shared" si="3"/>
+        <v>3.32</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>10</v>
       </c>
@@ -3058,8 +5707,20 @@
       <c r="E55" s="18">
         <v>3142</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F55">
+        <f t="shared" si="1"/>
+        <v>0.92</v>
+      </c>
+      <c r="G55">
+        <f t="shared" si="2"/>
+        <v>2.75</v>
+      </c>
+      <c r="H55">
+        <f t="shared" si="3"/>
+        <v>2.75</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>12</v>
       </c>
@@ -3075,8 +5736,20 @@
       <c r="E56" s="18">
         <v>1950</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F56">
+        <f t="shared" si="1"/>
+        <v>1.05</v>
+      </c>
+      <c r="G56">
+        <f t="shared" si="2"/>
+        <v>3.16</v>
+      </c>
+      <c r="H56">
+        <f t="shared" si="3"/>
+        <v>3.16</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>13</v>
       </c>
@@ -3092,8 +5765,20 @@
       <c r="E57" s="18">
         <v>900</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F57">
+        <f t="shared" si="1"/>
+        <v>0.77</v>
+      </c>
+      <c r="G57">
+        <f t="shared" si="2"/>
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="H57">
+        <f t="shared" si="3"/>
+        <v>2.2999999999999998</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>19</v>
       </c>
@@ -3109,8 +5794,20 @@
       <c r="E58" s="18">
         <v>1486</v>
       </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="F58">
+        <f t="shared" si="1"/>
+        <v>0.69</v>
+      </c>
+      <c r="G58">
+        <f t="shared" si="2"/>
+        <v>2.0699999999999998</v>
+      </c>
+      <c r="H58">
+        <f t="shared" si="3"/>
+        <v>2.0699999999999998</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>24</v>
       </c>
@@ -3125,6 +5822,18 @@
       </c>
       <c r="E59" s="18">
         <v>2744</v>
+      </c>
+      <c r="F59">
+        <f t="shared" si="1"/>
+        <v>1.17</v>
+      </c>
+      <c r="G59">
+        <f t="shared" si="2"/>
+        <v>3.5</v>
+      </c>
+      <c r="H59">
+        <f t="shared" si="3"/>
+        <v>3.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>